<commit_message>
docs: add Windows download and real Plot Docs screenshots
Refresh bundled templates without legacy branding, add the Windows EXE download link, and include screenshots of every editor plus the local account flow.
</commit_message>
<xml_diff>
--- a/apps/shell/resources/templates/Budget Planner.xlsx
+++ b/apps/shell/resources/templates/Budget Planner.xlsx
@@ -1004,8 +1004,8 @@
   <pageMargins left="0.45" right="0.45" top="0.65" bottom="0.6" header="0.5" footer="0.5"/>
   <pageSetup orientation="portrait" fitToHeight="0" fitToWidth="1"/>
   <headerFooter>
-    <oddHeader>&amp;C&amp;9 &amp;K667085&amp;BPLOT DOCS SUITE&amp;"Calibri,Bold"  /  Budget Planner</oddHeader>
-    <oddFooter>&amp;L&amp;8 &amp;K667085Built with Plot Docs Suite&amp;R&amp;8 &amp;K667085Page &amp;P of &amp;N</oddFooter>
+    <oddHeader>&amp;C&amp;9 &amp;K667085&amp;BPLOT DOCS&amp;"Calibri,Bold"  /  Budget Planner</oddHeader>
+    <oddFooter>&amp;L&amp;8 &amp;K667085Built with Plot Docs&amp;R&amp;8 &amp;K667085Page &amp;P of &amp;N</oddFooter>
     <evenHeader/>
     <evenFooter/>
     <firstHeader/>
@@ -1098,8 +1098,8 @@
   <pageMargins left="0.45" right="0.45" top="0.65" bottom="0.6" header="0.5" footer="0.5"/>
   <pageSetup orientation="portrait" fitToHeight="0" fitToWidth="1"/>
   <headerFooter>
-    <oddHeader>&amp;C&amp;9 &amp;K667085&amp;BPLOT DOCS SUITE&amp;"Calibri,Bold"  /  Budget Planner · Guide</oddHeader>
-    <oddFooter>&amp;L&amp;8 &amp;K667085Built with Plot Docs Suite&amp;R&amp;8 &amp;K667085Page &amp;P of &amp;N</oddFooter>
+    <oddHeader>&amp;C&amp;9 &amp;K667085&amp;BPLOT DOCS&amp;"Calibri,Bold"  /  Budget Planner · Guide</oddHeader>
+    <oddFooter>&amp;L&amp;8 &amp;K667085Built with Plot Docs&amp;R&amp;8 &amp;K667085Page &amp;P of &amp;N</oddFooter>
     <evenHeader/>
     <evenFooter/>
     <firstHeader/>

</xml_diff>